<commit_message>
updated plots and added email functionality, add new party, added polls
</commit_message>
<xml_diff>
--- a/party-comparison-updated-v38.xlsx
+++ b/party-comparison-updated-v38.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="29580" yWindow="780" windowWidth="21600" windowHeight="11295" tabRatio="500" firstSheet="4" activeTab="4" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="0" activeTab="5" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="כל הרשימות" sheetId="1" state="visible" r:id="rId1"/>
@@ -47362,7 +47362,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5703125" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -47400,7 +47400,7 @@
         </is>
       </c>
       <c r="B2" s="11" t="n">
-        <v>25</v>
+        <v>22.9</v>
       </c>
       <c r="C2" s="10">
         <f>ROUND(B2,0)</f>
@@ -47418,7 +47418,7 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>23.8</v>
+        <v>24.2</v>
       </c>
       <c r="C3" s="10">
         <f>ROUND(B3,0)</f>
@@ -47436,7 +47436,7 @@
         </is>
       </c>
       <c r="B4" s="11" t="n">
-        <v>12</v>
+        <v>13.3</v>
       </c>
       <c r="C4" s="10">
         <f>ROUND(B4,0)</f>
@@ -47472,7 +47472,7 @@
         </is>
       </c>
       <c r="B6" s="11" t="n">
-        <v>9.199999999999999</v>
+        <v>9.4</v>
       </c>
       <c r="C6" s="10">
         <f>ROUND(B6,0)</f>
@@ -47490,7 +47490,7 @@
         </is>
       </c>
       <c r="B7" s="11" t="n">
-        <v>8.4</v>
+        <v>7.5</v>
       </c>
       <c r="C7" s="10">
         <f>ROUND(B7,0)</f>
@@ -47508,7 +47508,7 @@
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>8.1</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C8" s="10">
         <f>ROUND(B8,0)</f>
@@ -47544,7 +47544,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>1.2</v>
+        <v>2.2</v>
       </c>
       <c r="C10" s="10">
         <f>ROUND(B10,0)</f>
@@ -47562,7 +47562,7 @@
         </is>
       </c>
       <c r="B11" s="11" t="n">
-        <v>4.9</v>
+        <v>4.7</v>
       </c>
       <c r="C11" s="10">
         <f>ROUND(B11,0)</f>
@@ -47580,7 +47580,7 @@
         </is>
       </c>
       <c r="B12" s="11" t="n">
-        <v>4.9</v>
+        <v>5</v>
       </c>
       <c r="C12" s="10">
         <f>ROUND(B12,0)</f>
@@ -47598,7 +47598,7 @@
         </is>
       </c>
       <c r="B13" s="11" t="n">
-        <v>2.6</v>
+        <v>2.7</v>
       </c>
       <c r="C13" s="10">
         <f>ROUND(B13,0)</f>
@@ -47616,7 +47616,7 @@
         </is>
       </c>
       <c r="B14" s="11" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="C14" s="10">
         <f>ROUND(B14,0)</f>
@@ -47660,6 +47660,24 @@
       </c>
       <c r="D16" s="10">
         <f>IF(C16&lt;=3,0,C16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>עמך ישראל</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C17">
+        <f>ROUND(B17,0)</f>
+        <v/>
+      </c>
+      <c r="D17">
+        <f>IF(C17&lt;=3,0,C17)</f>
         <v/>
       </c>
     </row>
@@ -47676,7 +47694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E204"/>
+  <dimension ref="A1:E215"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5703125" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -52755,6 +52773,281 @@
       <c r="E204" t="inlineStr">
         <is>
           <t>פריימריז</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>עמך ישראל</t>
+        </is>
+      </c>
+      <c r="B205" t="n">
+        <v>1</v>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>עופר וינטר</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>ז</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>מנהיג ומייסד המפלגה, תא"ל במיל'; הושקה 25.8.26 (ynet, ערוץ 7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>עמך ישראל</t>
+        </is>
+      </c>
+      <c r="B206" t="n">
+        <v>2</v>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>יוסף חדאד</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>ז</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>פעיל הסברה, מס' 2 ברשימה (הוכרז במפורש); ערוץ 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>עמך ישראל</t>
+        </is>
+      </c>
+      <c r="B207" t="n">
+        <v>3</v>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>נטעלי שם טוב</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>נ</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>עיתונאית ומגישת חדשות; ערוץ 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>עמך ישראל</t>
+        </is>
+      </c>
+      <c r="B208" t="n">
+        <v>4</v>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>סיגל קראוניק-עטיה</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>נ</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>אלמנת רבש"ץ בארי אריק קראוניק ז"ל; ערוץ 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>עמך ישראל</t>
+        </is>
+      </c>
+      <c r="B209" t="n">
+        <v>5</v>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>ללי דרעי</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>נ</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>אם שכולה (בנה נפל בעזה, יוני 2024); ערוץ 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>עמך ישראל</t>
+        </is>
+      </c>
+      <c r="B210" t="n">
+        <v>6</v>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>דוידי בן ציון</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>ז</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>סגן ומ"מ ראש המועצה האזורית שומרון; ערוץ 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>עמך ישראל</t>
+        </is>
+      </c>
+      <c r="B211" t="n">
+        <v>7</v>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>אלי ג'ינו</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>ז</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>אל"ם במיל', מפקד סיירת גבעתי לשעבר; ערוץ 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>עמך ישראל</t>
+        </is>
+      </c>
+      <c r="B212" t="n">
+        <v>8</v>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>ערן בן-ארי</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>ז</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>עו"ד, חבר המועצה הארצית ומוביל האופוזיציה בלשכת עוה"ד; ערוץ 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>עמך ישראל</t>
+        </is>
+      </c>
+      <c r="B213" t="n">
+        <v>9</v>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>פלר חסן-נחום</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>נ</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>עו"ד, לשעבר משנה לראש עיריית ירושלים; ערוץ 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>עמך ישראל</t>
+        </is>
+      </c>
+      <c r="B214" t="n">
+        <v>10</v>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>רונן בודנרו</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>ז</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>כלכלן; ערוץ 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>עמך ישראל</t>
+        </is>
+      </c>
+      <c r="B215" t="n">
+        <v>11</v>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>אביב עזרא</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>ז</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>מייסד ויו"ר תנועת "דור הניצחון"; ערוץ 7</t>
         </is>
       </c>
     </row>
@@ -52776,7 +53069,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5703125" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -53386,37 +53679,75 @@
       <c r="I16" s="15" t="n"/>
     </row>
     <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="12" t="inlineStr">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>עמך ישראל</t>
+        </is>
+      </c>
+      <c r="B17">
+        <f>INDEX('סקר 2026'!$D:$D,MATCH(A17,'סקר 2026'!$A:$A,0))</f>
+        <v/>
+      </c>
+      <c r="C17">
+        <f>COUNTIFS('מועמדים 2026'!$A:$A,A17,'מועמדים 2026'!$D:$D,"נ",'מועמדים 2026'!$B:$B,"&lt;="&amp;B17)</f>
+        <v/>
+      </c>
+      <c r="D17">
+        <f>COUNTIFS('מועמדים 2026'!$A:$A,A17,'מועמדים 2026'!$D:$D,"ז",'מועמדים 2026'!$B:$B,"&lt;="&amp;B17)</f>
+        <v/>
+      </c>
+      <c r="E17">
+        <f>IF(B17=0,0,C17/B17)</f>
+        <v/>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>מפלגה חדשה, הוקמה ע"י תא"ל (במיל') עופר וינטר; הושקה רשמית ב-25.8.2026. רשימה מבוססת דיווחי תקשורת ממסיבת ההשקה (ynet, ערוץ 7) - רשימה סופית וממוספרת רשמית טרם פורסמה לוועדת הבחירות המרכזית.</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17">
+        <f>IF(G17=0,0,H17/G17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
         <is>
           <t>סה"כ</t>
         </is>
       </c>
-      <c r="B17" s="12">
-        <f>SUM(B2:B16)</f>
-        <v/>
-      </c>
-      <c r="C17" s="12">
-        <f>SUM(C2:C16)</f>
-        <v/>
-      </c>
-      <c r="D17" s="12">
-        <f>SUM(D2:D16)</f>
-        <v/>
-      </c>
-      <c r="E17" s="16">
-        <f>IF(B17=0,0,C17/B17)</f>
-        <v/>
-      </c>
-      <c r="G17">
-        <f>SUM(G2:G16)</f>
-        <v/>
-      </c>
-      <c r="H17">
-        <f>SUM(H2:H16)</f>
-        <v/>
-      </c>
-      <c r="I17" s="15">
-        <f>IF(G17=0,0,H17/G17)</f>
+      <c r="B18" s="12">
+        <f>SUM(B2:B17)</f>
+        <v/>
+      </c>
+      <c r="C18" s="12">
+        <f>SUM(C2:C17)</f>
+        <v/>
+      </c>
+      <c r="D18" s="12">
+        <f>SUM(D2:D17)</f>
+        <v/>
+      </c>
+      <c r="E18" s="16">
+        <f>IF(B18=0,0,C18/B18)</f>
+        <v/>
+      </c>
+      <c r="G18">
+        <f>SUM(G2:G17)</f>
+        <v/>
+      </c>
+      <c r="H18">
+        <f>SUM(H2:H17)</f>
+        <v/>
+      </c>
+      <c r="I18" s="15">
+        <f>IF(G18=0,0,H18/G18)</f>
         <v/>
       </c>
     </row>
@@ -57814,7 +58145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R11"/>
+  <dimension ref="A1:S11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -57908,37 +58239,45 @@
           <t>האחדות</t>
         </is>
       </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>עמך ישראל</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>חדשות 12</t>
+          <t>וואלה</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>מנו גבע</t>
+          <t>מנחם לזר</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>502</t>
+          <t>500</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G2" t="n">
         <v>7</v>
       </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
       <c r="I2" t="n">
         <v>7</v>
       </c>
@@ -57946,28 +58285,37 @@
         <v>9</v>
       </c>
       <c r="K2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="L2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="O2" t="n">
         <v>15</v>
       </c>
       <c r="P2" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ערוץ 14</t>
+          <t>חדשות 12</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -57977,43 +58325,43 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>שלמה פילבר</t>
+          <t>מנו גבע</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>486</t>
+          <t>502</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="F3" t="n">
         <v>8</v>
       </c>
       <c r="G3" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="I3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J3" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K3" t="n">
+        <v>11</v>
+      </c>
+      <c r="L3" t="n">
+        <v>4</v>
+      </c>
+      <c r="M3" t="n">
+        <v>4</v>
+      </c>
+      <c r="N3" t="n">
         <v>9</v>
       </c>
-      <c r="L3" t="n">
-        <v>5</v>
-      </c>
-      <c r="M3" t="n">
-        <v>5</v>
-      </c>
-      <c r="N3" t="n">
-        <v>8</v>
-      </c>
       <c r="O3" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="P3" t="n">
         <v>24</v>
@@ -58022,44 +58370,41 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>כאן חדשות</t>
+          <t>ערוץ 14</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>דודי חסיד</t>
+          <t>שלמה פילבר</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>552</t>
+          <t>486</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="F4" t="n">
         <v>8</v>
       </c>
       <c r="G4" t="n">
+        <v>10</v>
+      </c>
+      <c r="I4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J4" t="n">
         <v>7</v>
       </c>
-      <c r="H4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" t="n">
-        <v>7</v>
-      </c>
-      <c r="J4" t="n">
+      <c r="K4" t="n">
         <v>9</v>
-      </c>
-      <c r="K4" t="n">
-        <v>10</v>
       </c>
       <c r="L4" t="n">
         <v>5</v>
@@ -58068,44 +58413,38 @@
         <v>5</v>
       </c>
       <c r="N4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="O4" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="P4" t="n">
         <v>24</v>
       </c>
-      <c r="Q4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R4" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>מעריב</t>
+          <t>כאן חדשות</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>מנחם לזר</t>
+          <t>דודי חסיד</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>501</t>
+          <t>552</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F5" t="n">
         <v>8</v>
@@ -58113,11 +58452,14 @@
       <c r="G5" t="n">
         <v>7</v>
       </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
       <c r="I5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J5" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K5" t="n">
         <v>10</v>
@@ -58135,32 +58477,41 @@
         <v>14</v>
       </c>
       <c r="P5" t="n">
-        <v>26</v>
+        <v>24</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ישראל היום</t>
+          <t>מעריב</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>דודי חסיד</t>
+          <t>מנחם לזר</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>553</t>
+          <t>501</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F6" t="n">
         <v>8</v>
@@ -58169,7 +58520,7 @@
         <v>7</v>
       </c>
       <c r="I6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J6" t="n">
         <v>10</v>
@@ -58187,16 +58538,16 @@
         <v>9</v>
       </c>
       <c r="O6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P6" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>זמן ישראל</t>
+          <t>ישראל היום</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -58206,43 +58557,43 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>יוסי טאטיקה</t>
+          <t>דודי חסיד</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>553</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F7" t="n">
         <v>8</v>
       </c>
       <c r="G7" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J7" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="K7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M7" t="n">
         <v>5</v>
       </c>
       <c r="N7" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="O7" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="P7" t="n">
         <v>23</v>
@@ -58251,62 +58602,62 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>חדשות 13</t>
+          <t>זמן ישראל</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>המדד</t>
+          <t>יוסי טאטיקה</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>961</t>
+          <t>400</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F8" t="n">
         <v>8</v>
       </c>
       <c r="G8" t="n">
+        <v>9</v>
+      </c>
+      <c r="I8" t="n">
         <v>7</v>
       </c>
-      <c r="I8" t="n">
-        <v>5</v>
-      </c>
       <c r="J8" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K8" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="L8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M8" t="n">
         <v>5</v>
       </c>
       <c r="N8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="O8" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="P8" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ערוץ 16</t>
+          <t>חדשות 13</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -58316,22 +58667,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>יצחק כ״ץ</t>
+          <t>המדד</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>961</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F9" t="n">
+        <v>8</v>
+      </c>
+      <c r="G9" t="n">
         <v>7</v>
-      </c>
-      <c r="G9" t="n">
-        <v>9</v>
       </c>
       <c r="I9" t="n">
         <v>5</v>
@@ -58340,112 +58691,109 @@
         <v>9</v>
       </c>
       <c r="K9" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="O9" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="P9" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>i24 news</t>
+          <t>ערוץ 16</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>דירקט פולס</t>
+          <t>יצחק כ״ץ</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>522</t>
+          <t>500</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="F10" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I10" t="n">
         <v>5</v>
       </c>
       <c r="J10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K10" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="L10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N10" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="O10" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="P10" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>וואלה</t>
+          <t>i24 news</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>מנחם לזר</t>
+          <t>דירקט פולס</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>522</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F11" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G11" t="n">
         <v>8</v>
       </c>
-      <c r="H11" t="n">
-        <v>0</v>
-      </c>
       <c r="I11" t="n">
         <v>5</v>
       </c>
@@ -58453,25 +58801,22 @@
         <v>8</v>
       </c>
       <c r="K11" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="L11" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="M11" t="n">
         <v>5</v>
       </c>
       <c r="N11" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O11" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="P11" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>